<commit_message>
nog meer naam veranderingen
</commit_message>
<xml_diff>
--- a/baseline_code/Data/Plane_data.xlsx
+++ b/baseline_code/Data/Plane_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="34">
   <si>
     <t>Plane</t>
   </si>
@@ -25,6 +25,12 @@
     <t>SIBT</t>
   </si>
   <si>
+    <t>Cargo From</t>
+  </si>
+  <si>
+    <t>Cargo To</t>
+  </si>
+  <si>
     <t>KL642</t>
   </si>
   <si>
@@ -34,12 +40,21 @@
     <t>120</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>BA441</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>LH997</t>
   </si>
   <si>
@@ -47,6 +62,9 @@
   </si>
   <si>
     <t>150</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
   <si>
     <t>AF1341</t>
@@ -469,10 +487,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,115 +500,181 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E10" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
         <v>12</v>
       </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
+      <c r="E11" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Realistic drive speed, smooth driving of GSEs
</commit_message>
<xml_diff>
--- a/baseline_code/Data/Plane_data.xlsx
+++ b/baseline_code/Data/Plane_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="36">
   <si>
     <t>Plane</t>
   </si>
@@ -43,6 +43,11 @@
     <t>1</t>
   </si>
   <si>
+    <r>
+      <t>4</t>
+    </r>
+  </si>
+  <si>
     <t>BA441</t>
   </si>
   <si>
@@ -61,7 +66,14 @@
     <t>9</t>
   </si>
   <si>
-    <t>150</t>
+    <r>
+      <t>15</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3</t>
+    </r>
   </si>
   <si>
     <t>4</t>
@@ -521,157 +533,157 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
       <c r="E5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>

</xml_diff>